<commit_message>
data: pin Sdp headers to camelCase via [ColumnName] -> byte-identical to committed CSVs (Sdp is drop-in generator, zero Unity change); camelCase authoring workbook
</commit_message>
<xml_diff>
--- a/Assets/_Tower/Data/Source/Tower_GameData.xlsx
+++ b/Assets/_Tower/Data/Source/Tower_GameData.xlsx
@@ -424,22 +424,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>DisplayName</t>
+          <t>displayName</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>DurationTurns</t>
+          <t>durationTurns</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Stackable</t>
+          <t>stackable</t>
         </is>
       </c>
     </row>
@@ -504,17 +504,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>DisplayName</t>
+          <t>displayName</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>EffectHookKey</t>
+          <t>effectHookKey</t>
         </is>
       </c>
     </row>
@@ -586,52 +586,52 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>DisplayName</t>
+          <t>displayName</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>tag</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>TargetMark</t>
+          <t>targetMark</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>range</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>cost</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>BasePower</t>
+          <t>basePower</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>AmplificationMultiplier</t>
+          <t>amplificationMultiplier</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>TargetType</t>
+          <t>targetType</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>CooldownRounds</t>
+          <t>cooldownRounds</t>
         </is>
       </c>
     </row>
@@ -1152,67 +1152,67 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>DisplayName</t>
+          <t>displayName</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>MaxHp</t>
+          <t>maxHp</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Attack</t>
+          <t>attack</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Defense</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>speed</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Disposition</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Passive</t>
+          <t>passive</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>DefaultAbilities</t>
+          <t>defaultAbilities</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>IsReturner</t>
+          <t>isReturner</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>ChainLocked</t>
+          <t>chainLocked</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>IsPreset</t>
+          <t>isPreset</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>FactionId</t>
+          <t>factionId</t>
         </is>
       </c>
     </row>
@@ -1501,32 +1501,32 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>DisplayName</t>
+          <t>displayName</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>ResourceScope</t>
+          <t>resourceScope</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>power</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>StackMax</t>
+          <t>stackMax</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>description</t>
         </is>
       </c>
     </row>
@@ -1611,37 +1611,37 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>TableId</t>
+          <t>tableId</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>EntryId</t>
+          <t>entryId</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Weight</t>
+          <t>weight</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>RewardType</t>
+          <t>rewardType</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>RefId</t>
+          <t>refId</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>MinDepth</t>
+          <t>minDepth</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>MaxDepth</t>
+          <t>maxDepth</t>
         </is>
       </c>
     </row>

</xml_diff>